<commit_message>
feat: update viva grading mark sheet with new course details and formatting
</commit_message>
<xml_diff>
--- a/Viva_Grading_Mark_sheet.xlsx
+++ b/Viva_Grading_Mark_sheet.xlsx
@@ -7,8 +7,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mark Guide" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SE2040 Marks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DS1030 Marks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SE3010 Marks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IT2040 Marks" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1185,7 +1185,7 @@
     <row r="1" ht="18" customHeight="1" s="11">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>SE2040 - Software Testing: expert mark and system mark</t>
+          <t>SE3010 - Software Engineering Process &amp; Quality Management</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
     <row r="1" ht="18" customHeight="1" s="11">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>DS1030 - ER Modelling: expert mark and system mark</t>
+          <t>IT2040 - Database Management Systems (DBMS)</t>
         </is>
       </c>
     </row>

</xml_diff>